<commit_message>
Refactor analysis scripts and update Excel outputs
- Updated `printing_all_flags.ipynb` to comment out CSV reading and related operations.
- Added new script `sort_records_by_amount_of_extrasystols.ipynb` for sorting records based on specified criteria.
- Created new Excel files: `sorted_visi_zive_irasai_atrankai._extended.xlsx` and `visi_zive_irasai_atrankai._extended_sorted_grouped_highlighted.xlsx` for sorted and highlighted outputs.
- Adjusted noise annotation indices in `04_SarasasTriuksmuZymejimui .txt`.
- Updated `records_summary_zymetas.xlsx` with new data.
</commit_message>
<xml_diff>
--- a/1_PREPARE_TRAIN_UNET_DATA/TriuksmaiAnotacijosDuomenyse2023/records_summary_zymetas.xlsx
+++ b/1_PREPARE_TRAIN_UNET_DATA/TriuksmaiAnotacijosDuomenyse2023/records_summary_zymetas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\1_PREPARE_TRAIN_UNET_DATA\TriuksmaiAnotacijosDuomenyse2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00D9B02-62C6-4B83-BE91-F6900F1FF70D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701388DB-8DDE-41F9-A1CD-3FF5A3EFEEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="151">
   <si>
     <t>nr</t>
   </si>
@@ -471,6 +471,9 @@
   </si>
   <si>
     <t>Nika</t>
+  </si>
+  <si>
+    <t>['AI_DATASET' ,'FULLY_ANNOTATED_PROFESSIONALLY','NOISES_ANNOTATED']</t>
   </si>
 </sst>
 </file>
@@ -872,7 +875,7 @@
     <col min="4" max="4" width="12.453125" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="13.26953125" customWidth="1"/>
-    <col min="7" max="7" width="52.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="67.36328125" customWidth="1"/>
     <col min="8" max="8" width="25.26953125" customWidth="1"/>
     <col min="9" max="9" width="25.1796875" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="7.6328125" hidden="1" customWidth="1"/>
@@ -967,7 +970,7 @@
         <v>20</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="H2" t="s">
         <v>21</v>
@@ -1026,7 +1029,7 @@
         <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="H3" t="s">
         <v>26</v>
@@ -1085,7 +1088,7 @@
         <v>28</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="H4" t="s">
         <v>29</v>
@@ -1144,7 +1147,7 @@
         <v>32</v>
       </c>
       <c r="G5" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="H5" t="s">
         <v>33</v>
@@ -1203,7 +1206,7 @@
         <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="H6" t="s">
         <v>37</v>
@@ -1262,7 +1265,7 @@
         <v>39</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="H7" t="s">
         <v>40</v>
@@ -1321,7 +1324,7 @@
         <v>43</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>150</v>
       </c>
       <c r="H8" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
Add new script to convert ZIVE format files to .npy and update records summary Excel file
</commit_message>
<xml_diff>
--- a/1_PREPARE_TRAIN_UNET_DATA/TriuksmaiAnotacijosDuomenyse2023/records_summary_zymetas.xlsx
+++ b/1_PREPARE_TRAIN_UNET_DATA/TriuksmaiAnotacijosDuomenyse2023/records_summary_zymetas.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\1_PREPARE_TRAIN_UNET_DATA\TriuksmaiAnotacijosDuomenyse2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701388DB-8DDE-41F9-A1CD-3FF5A3EFEEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5CB7D70-203B-4606-83FD-DA6CD3B4F262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Svaruoliai" sheetId="1" r:id="rId1"/>
     <sheet name="Triuksmuoliai" sheetId="2" r:id="rId2"/>
+    <sheet name="Ypatingi" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="159">
   <si>
     <t>nr</t>
   </si>
@@ -92,9 +93,6 @@
     <t>60a917b354352a3df86dc1f2</t>
   </si>
   <si>
-    <t>['FULLY_ANNOTATED_PROFESSIONALLY']</t>
-  </si>
-  <si>
     <t>1001_8.npy</t>
   </si>
   <si>
@@ -474,6 +472,33 @@
   </si>
   <si>
     <t>['AI_DATASET' ,'FULLY_ANNOTATED_PROFESSIONALLY','NOISES_ANNOTATED']</t>
+  </si>
+  <si>
+    <t>FULLY_ANNOTATED_PROFESSIONALLY</t>
+  </si>
+  <si>
+    <t>AI_DATASET</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>1740295.071</t>
+  </si>
+  <si>
+    <t>1742295.469</t>
+  </si>
+  <si>
+    <t>1742319.328</t>
+  </si>
+  <si>
+    <t>1742362.474</t>
+  </si>
+  <si>
+    <t>Igno Griskeviciaus su nepagautomis V</t>
+  </si>
+  <si>
+    <t>Žygimantas</t>
   </si>
 </sst>
 </file>
@@ -484,7 +509,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -502,6 +527,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF6A9955"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -551,7 +588,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -564,6 +601,18 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -896,7 +945,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
@@ -958,7 +1007,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D2" s="6" t="b">
         <v>1</v>
@@ -970,7 +1019,7 @@
         <v>20</v>
       </c>
       <c r="G2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H2" t="s">
         <v>21</v>
@@ -1017,22 +1066,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D3" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
         <v>24</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>149</v>
+      </c>
+      <c r="H3" t="s">
         <v>25</v>
-      </c>
-      <c r="G3" t="s">
-        <v>150</v>
-      </c>
-      <c r="H3" t="s">
-        <v>26</v>
       </c>
       <c r="I3" t="s">
         <v>22</v>
@@ -1076,25 +1125,25 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D4" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
         <v>27</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
+        <v>149</v>
+      </c>
+      <c r="H4" t="s">
         <v>28</v>
       </c>
-      <c r="G4" t="s">
-        <v>150</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>29</v>
-      </c>
-      <c r="I4" t="s">
-        <v>30</v>
       </c>
       <c r="J4">
         <v>127999</v>
@@ -1135,25 +1184,25 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D5" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s">
         <v>31</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
+        <v>149</v>
+      </c>
+      <c r="H5" t="s">
         <v>32</v>
       </c>
-      <c r="G5" t="s">
-        <v>150</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>33</v>
-      </c>
-      <c r="I5" t="s">
-        <v>34</v>
       </c>
       <c r="J5">
         <v>127999</v>
@@ -1194,25 +1243,25 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D6" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
         <v>35</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
+        <v>149</v>
+      </c>
+      <c r="H6" t="s">
         <v>36</v>
       </c>
-      <c r="G6" t="s">
-        <v>150</v>
-      </c>
-      <c r="H6" t="s">
-        <v>37</v>
-      </c>
       <c r="I6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J6">
         <v>127999</v>
@@ -1253,25 +1302,25 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D7" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" t="s">
         <v>38</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
+        <v>149</v>
+      </c>
+      <c r="H7" t="s">
         <v>39</v>
       </c>
-      <c r="G7" t="s">
-        <v>150</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>40</v>
-      </c>
-      <c r="I7" t="s">
-        <v>41</v>
       </c>
       <c r="J7">
         <v>127999</v>
@@ -1312,25 +1361,25 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D8" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" t="s">
         <v>42</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>149</v>
+      </c>
+      <c r="H8" t="s">
         <v>43</v>
       </c>
-      <c r="G8" t="s">
-        <v>150</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>44</v>
-      </c>
-      <c r="I8" t="s">
-        <v>45</v>
       </c>
       <c r="J8">
         <v>127999</v>
@@ -1371,25 +1420,25 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>149</v>
-      </c>
-      <c r="C9" s="7" t="b">
+        <v>148</v>
+      </c>
+      <c r="D9" s="7" t="b">
         <v>1</v>
       </c>
       <c r="E9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" t="s">
         <v>46</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
+        <v>149</v>
+      </c>
+      <c r="H9" t="s">
         <v>47</v>
       </c>
-      <c r="G9" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>48</v>
-      </c>
-      <c r="I9" t="s">
-        <v>49</v>
       </c>
       <c r="J9">
         <v>127999</v>
@@ -1430,25 +1479,25 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>149</v>
-      </c>
-      <c r="C10" s="7" t="b">
+        <v>148</v>
+      </c>
+      <c r="D10" s="7" t="b">
         <v>1</v>
       </c>
       <c r="E10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" t="s">
         <v>50</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
+        <v>149</v>
+      </c>
+      <c r="H10" t="s">
         <v>51</v>
       </c>
-      <c r="G10" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" t="s">
-        <v>52</v>
-      </c>
       <c r="I10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J10">
         <v>127999</v>
@@ -1489,25 +1538,25 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>149</v>
-      </c>
-      <c r="C11" s="7" t="b">
+        <v>148</v>
+      </c>
+      <c r="D11" s="7" t="b">
         <v>1</v>
       </c>
       <c r="E11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" t="s">
         <v>53</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
+        <v>149</v>
+      </c>
+      <c r="H11" t="s">
         <v>54</v>
       </c>
-      <c r="G11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>55</v>
-      </c>
-      <c r="I11" t="s">
-        <v>56</v>
       </c>
       <c r="J11">
         <v>127999</v>
@@ -1548,25 +1597,25 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>149</v>
-      </c>
-      <c r="C12" s="7" t="b">
+        <v>148</v>
+      </c>
+      <c r="D12" s="7" t="b">
         <v>1</v>
       </c>
       <c r="E12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" t="s">
         <v>57</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
+        <v>149</v>
+      </c>
+      <c r="H12" t="s">
         <v>58</v>
       </c>
-      <c r="G12" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12" t="s">
-        <v>59</v>
-      </c>
       <c r="I12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J12">
         <v>127999</v>
@@ -1607,25 +1656,25 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D13" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" t="s">
         <v>60</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
+        <v>149</v>
+      </c>
+      <c r="H13" t="s">
         <v>61</v>
       </c>
-      <c r="G13" t="s">
-        <v>23</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>62</v>
-      </c>
-      <c r="I13" t="s">
-        <v>63</v>
       </c>
       <c r="J13">
         <v>127999</v>
@@ -1666,25 +1715,25 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D14" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" t="s">
         <v>64</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
+        <v>149</v>
+      </c>
+      <c r="H14" t="s">
         <v>65</v>
       </c>
-      <c r="G14" t="s">
-        <v>23</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>66</v>
-      </c>
-      <c r="I14" t="s">
-        <v>67</v>
       </c>
       <c r="J14">
         <v>127999</v>
@@ -1725,25 +1774,25 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D15" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15" t="s">
         <v>68</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
+        <v>149</v>
+      </c>
+      <c r="H15" t="s">
         <v>69</v>
       </c>
-      <c r="G15" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" t="s">
-        <v>70</v>
-      </c>
       <c r="I15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J15">
         <v>127999</v>
@@ -1784,25 +1833,25 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D16" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" t="s">
         <v>71</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
+        <v>149</v>
+      </c>
+      <c r="H16" t="s">
         <v>72</v>
       </c>
-      <c r="G16" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>73</v>
-      </c>
-      <c r="I16" t="s">
-        <v>74</v>
       </c>
       <c r="J16">
         <v>127999</v>
@@ -1843,25 +1892,25 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D17" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E17" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" t="s">
         <v>75</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
+        <v>149</v>
+      </c>
+      <c r="H17" t="s">
         <v>76</v>
       </c>
-      <c r="G17" t="s">
-        <v>23</v>
-      </c>
-      <c r="H17" t="s">
-        <v>77</v>
-      </c>
       <c r="I17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J17">
         <v>127999</v>
@@ -1902,25 +1951,25 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D18" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E18" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" t="s">
         <v>78</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
+        <v>149</v>
+      </c>
+      <c r="H18" t="s">
         <v>79</v>
       </c>
-      <c r="G18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>80</v>
-      </c>
-      <c r="I18" t="s">
-        <v>81</v>
       </c>
       <c r="J18">
         <v>127999</v>
@@ -1961,25 +2010,25 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>149</v>
-      </c>
-      <c r="C19" s="7" t="b">
+        <v>148</v>
+      </c>
+      <c r="D19" s="7" t="b">
         <v>1</v>
       </c>
       <c r="E19" t="s">
+        <v>81</v>
+      </c>
+      <c r="F19" t="s">
         <v>82</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
+        <v>149</v>
+      </c>
+      <c r="H19" t="s">
         <v>83</v>
       </c>
-      <c r="G19" t="s">
-        <v>23</v>
-      </c>
-      <c r="H19" t="s">
-        <v>84</v>
-      </c>
       <c r="I19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J19">
         <v>127999</v>
@@ -2020,25 +2069,25 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D20" s="5" t="b">
         <v>1</v>
       </c>
       <c r="E20" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" t="s">
         <v>85</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
+        <v>149</v>
+      </c>
+      <c r="H20" t="s">
         <v>86</v>
       </c>
-      <c r="G20" t="s">
-        <v>23</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>87</v>
-      </c>
-      <c r="I20" t="s">
-        <v>88</v>
       </c>
       <c r="J20">
         <v>127999</v>
@@ -2079,25 +2128,25 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D21" s="5" t="b">
         <v>1</v>
       </c>
       <c r="E21" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" t="s">
         <v>89</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
+        <v>149</v>
+      </c>
+      <c r="H21" t="s">
         <v>90</v>
       </c>
-      <c r="G21" t="s">
-        <v>23</v>
-      </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>91</v>
-      </c>
-      <c r="I21" t="s">
-        <v>92</v>
       </c>
       <c r="J21">
         <v>127999</v>
@@ -2138,25 +2187,25 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D22" s="5" t="b">
         <v>1</v>
       </c>
       <c r="E22" t="s">
+        <v>92</v>
+      </c>
+      <c r="F22" t="s">
         <v>93</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
+        <v>149</v>
+      </c>
+      <c r="H22" t="s">
         <v>94</v>
       </c>
-      <c r="G22" t="s">
-        <v>23</v>
-      </c>
-      <c r="H22" t="s">
-        <v>95</v>
-      </c>
       <c r="I22" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J22">
         <v>127999</v>
@@ -2197,25 +2246,25 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D23" s="5" t="b">
         <v>1</v>
       </c>
       <c r="E23" t="s">
+        <v>95</v>
+      </c>
+      <c r="F23" t="s">
         <v>96</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
+        <v>149</v>
+      </c>
+      <c r="H23" t="s">
         <v>97</v>
       </c>
-      <c r="G23" t="s">
-        <v>23</v>
-      </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>98</v>
-      </c>
-      <c r="I23" t="s">
-        <v>99</v>
       </c>
       <c r="J23">
         <v>127999</v>
@@ -2256,25 +2305,25 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D24" s="5" t="b">
         <v>1</v>
       </c>
       <c r="E24" t="s">
+        <v>99</v>
+      </c>
+      <c r="F24" t="s">
         <v>100</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
+        <v>149</v>
+      </c>
+      <c r="H24" t="s">
         <v>101</v>
       </c>
-      <c r="G24" t="s">
-        <v>23</v>
-      </c>
-      <c r="H24" t="s">
-        <v>102</v>
-      </c>
       <c r="I24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J24">
         <v>127999</v>
@@ -2315,25 +2364,25 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D25" s="5" t="b">
         <v>1</v>
       </c>
       <c r="E25" t="s">
+        <v>102</v>
+      </c>
+      <c r="F25" t="s">
         <v>103</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
+        <v>149</v>
+      </c>
+      <c r="H25" t="s">
         <v>104</v>
       </c>
-      <c r="G25" t="s">
-        <v>23</v>
-      </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>105</v>
-      </c>
-      <c r="I25" t="s">
-        <v>106</v>
       </c>
       <c r="J25">
         <v>127999</v>
@@ -2374,25 +2423,25 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D26" s="5" t="b">
         <v>1</v>
       </c>
       <c r="E26" t="s">
+        <v>106</v>
+      </c>
+      <c r="F26" t="s">
         <v>107</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
+        <v>149</v>
+      </c>
+      <c r="H26" t="s">
         <v>108</v>
       </c>
-      <c r="G26" t="s">
-        <v>23</v>
-      </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>109</v>
-      </c>
-      <c r="I26" t="s">
-        <v>110</v>
       </c>
       <c r="J26">
         <v>127999</v>
@@ -2433,25 +2482,25 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>149</v>
-      </c>
-      <c r="C27" s="7" t="b">
+        <v>148</v>
+      </c>
+      <c r="D27" s="7" t="b">
         <v>1</v>
       </c>
       <c r="E27" t="s">
+        <v>110</v>
+      </c>
+      <c r="F27" t="s">
         <v>111</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
+        <v>149</v>
+      </c>
+      <c r="H27" t="s">
         <v>112</v>
       </c>
-      <c r="G27" t="s">
-        <v>23</v>
-      </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>113</v>
-      </c>
-      <c r="I27" t="s">
-        <v>114</v>
       </c>
       <c r="J27">
         <v>127999</v>
@@ -2492,25 +2541,25 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D28" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E28" t="s">
+        <v>114</v>
+      </c>
+      <c r="F28" t="s">
         <v>115</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
+        <v>149</v>
+      </c>
+      <c r="H28" t="s">
         <v>116</v>
       </c>
-      <c r="G28" t="s">
-        <v>23</v>
-      </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>117</v>
-      </c>
-      <c r="I28" t="s">
-        <v>118</v>
       </c>
       <c r="J28">
         <v>127999</v>
@@ -2551,25 +2600,25 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D29" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E29" t="s">
+        <v>118</v>
+      </c>
+      <c r="F29" t="s">
         <v>119</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
+        <v>149</v>
+      </c>
+      <c r="H29" t="s">
         <v>120</v>
       </c>
-      <c r="G29" t="s">
-        <v>23</v>
-      </c>
-      <c r="H29" t="s">
-        <v>121</v>
-      </c>
       <c r="I29" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J29">
         <v>127999</v>
@@ -2610,25 +2659,25 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D30" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E30" t="s">
+        <v>121</v>
+      </c>
+      <c r="F30" t="s">
         <v>122</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
+        <v>149</v>
+      </c>
+      <c r="H30" t="s">
         <v>123</v>
       </c>
-      <c r="G30" t="s">
-        <v>23</v>
-      </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>124</v>
-      </c>
-      <c r="I30" t="s">
-        <v>125</v>
       </c>
       <c r="J30">
         <v>127999</v>
@@ -2669,25 +2718,25 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D31" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E31" t="s">
+        <v>125</v>
+      </c>
+      <c r="F31" t="s">
         <v>126</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
+        <v>149</v>
+      </c>
+      <c r="H31" t="s">
         <v>127</v>
       </c>
-      <c r="G31" t="s">
-        <v>23</v>
-      </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>128</v>
-      </c>
-      <c r="I31" t="s">
-        <v>129</v>
       </c>
       <c r="J31">
         <v>127999</v>
@@ -2728,25 +2777,25 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D32" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E32" t="s">
+        <v>129</v>
+      </c>
+      <c r="F32" t="s">
         <v>130</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
+        <v>149</v>
+      </c>
+      <c r="H32" t="s">
         <v>131</v>
       </c>
-      <c r="G32" t="s">
-        <v>23</v>
-      </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
         <v>132</v>
-      </c>
-      <c r="I32" t="s">
-        <v>133</v>
       </c>
       <c r="J32">
         <v>127999</v>
@@ -2787,25 +2836,25 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D33" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E33" t="s">
+        <v>133</v>
+      </c>
+      <c r="F33" t="s">
         <v>134</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
+        <v>149</v>
+      </c>
+      <c r="H33" t="s">
         <v>135</v>
       </c>
-      <c r="G33" t="s">
-        <v>23</v>
-      </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>136</v>
-      </c>
-      <c r="I33" t="s">
-        <v>137</v>
       </c>
       <c r="J33">
         <v>127999</v>
@@ -2846,25 +2895,25 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D34" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E34" t="s">
+        <v>137</v>
+      </c>
+      <c r="F34" t="s">
         <v>138</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
+        <v>149</v>
+      </c>
+      <c r="H34" t="s">
         <v>139</v>
       </c>
-      <c r="G34" t="s">
-        <v>23</v>
-      </c>
-      <c r="H34" t="s">
-        <v>140</v>
-      </c>
       <c r="I34" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J34">
         <v>127999</v>
@@ -2905,25 +2954,25 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D35" s="6" t="b">
         <v>1</v>
       </c>
       <c r="E35" t="s">
+        <v>140</v>
+      </c>
+      <c r="F35" t="s">
         <v>141</v>
       </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
+        <v>149</v>
+      </c>
+      <c r="H35" t="s">
         <v>142</v>
       </c>
-      <c r="G35" t="s">
-        <v>23</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
         <v>143</v>
-      </c>
-      <c r="I35" t="s">
-        <v>144</v>
       </c>
       <c r="J35">
         <v>128000</v>
@@ -2967,19 +3016,19 @@
         <v>1</v>
       </c>
       <c r="E36" t="s">
+        <v>144</v>
+      </c>
+      <c r="F36" t="s">
         <v>145</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
+        <v>149</v>
+      </c>
+      <c r="H36" t="s">
         <v>146</v>
       </c>
-      <c r="G36" t="s">
-        <v>23</v>
-      </c>
-      <c r="H36" t="s">
-        <v>147</v>
-      </c>
       <c r="I36" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J36">
         <v>128000</v>
@@ -3027,4 +3076,178 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BE06B30-E83F-4AD8-A91F-4635C67152A2}">
+  <dimension ref="A1:V6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="11.36328125" customWidth="1"/>
+    <col min="3" max="3" width="21.54296875" customWidth="1"/>
+    <col min="4" max="4" width="25.81640625" customWidth="1"/>
+    <col min="5" max="5" width="21.26953125" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="12.6328125" customWidth="1"/>
+    <col min="8" max="8" width="40.453125" customWidth="1"/>
+    <col min="9" max="9" width="15.08984375" customWidth="1"/>
+    <col min="10" max="10" width="28.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C2" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="N2" s="3"/>
+      <c r="O2" s="2"/>
+      <c r="V2" s="3"/>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C3" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="N3" s="3"/>
+      <c r="O3" s="2"/>
+      <c r="V3" s="3"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="N4" s="3"/>
+      <c r="O4" s="2"/>
+      <c r="V4" s="3"/>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="C5" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="N5" s="3"/>
+      <c r="O5" s="2"/>
+      <c r="V5" s="3"/>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="2"/>
+      <c r="V6" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>